<commit_message>
refactor: remove schedule types and page components
- Deleted `schedule-types.ts` and `page.tsx` as part of the refactor to streamline the schedule management.
- Updated API for branding CSV exports to ensure sheet exports are handled correctly.
- Enhanced cross-wire print page to manage assignment visibility based on external locations.
- Improved switch component styles for better UI consistency.
- Added a script to map brand list names to project manifests, allowing for automated updates of project names based on file conventions.
- Introduced new API route for generating cross-wire PDFs.
</commit_message>
<xml_diff>
--- a/Share/Projects/ANG01_STOCK/exports/units/1/branding/ANG01 STOCK BRANDLIST A.6_M.2 #1 JB71 B,BOX CONTROL.xlsx
+++ b/Share/Projects/ANG01_STOCK/exports/units/1/branding/ANG01 STOCK BRANDLIST A.6_M.2 #1 JB71 B,BOX CONTROL.xlsx
@@ -33,7 +33,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -41,11 +41,6 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="13"/>
-      <name val="Calibri"/>
-      <b/>
     </font>
     <font>
       <sz val="13"/>
@@ -77,23 +72,8 @@
       <name val="Calibri"/>
       <b/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
   </fonts>
-  <fills count="11">
+  <fills count="8">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -112,25 +92,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF8FAFC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEEF2FF"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEEF2FF"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE2E8F0"/>
+        <fgColor rgb="FFE3E3E3"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -148,18 +110,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEEF2FF"/>
+        <fgColor rgb="FFF8FAFC"/>
         <bgColor/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEEF2FF"/>
+        <fgColor rgb="FFE3E3E3"/>
         <bgColor/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -174,43 +136,156 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="true"/>
     </xf>
   </cellXfs>
@@ -560,285 +635,285 @@
       <c r="A1" s="3" t="str">
         <v>JB71 B,BOX CONTROL</v>
       </c>
-      <c r="B1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H1" s="4" t="str">
+      <c r="B1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H1" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
-        <v/>
-      </c>
-      <c r="B2" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C2" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D2" s="2" t="str">
-        <v/>
-      </c>
-      <c r="E2" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F2" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G2" s="2" t="str">
-        <v/>
-      </c>
-      <c r="H2" s="2" t="str">
+      <c r="A2" s="4" t="str">
+        <v/>
+      </c>
+      <c r="B2" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C2" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D2" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E2" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F2" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G2" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H2" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
+      <c r="A3" s="4" t="str">
         <v>Project #</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="5" t="str">
         <v>ANG01</v>
       </c>
-      <c r="C3" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D3" s="2" t="str">
-        <v/>
-      </c>
-      <c r="E3" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F3" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G3" s="2" t="str">
-        <v/>
-      </c>
-      <c r="H3" s="2" t="str">
+      <c r="C3" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D3" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E3" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G3" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H3" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="str">
+      <c r="A4" s="4" t="str">
         <v>Project Name</v>
       </c>
-      <c r="B4" s="2" t="str">
+      <c r="B4" s="5" t="str">
         <v>STOCK</v>
       </c>
-      <c r="C4" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D4" s="2" t="str">
-        <v/>
-      </c>
-      <c r="E4" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F4" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G4" s="2" t="str">
-        <v/>
-      </c>
-      <c r="H4" s="2" t="str">
+      <c r="C4" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D4" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E4" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F4" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G4" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H4" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="str">
+      <c r="A5" s="4" t="str">
         <v>Revision</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="5" t="str">
         <v>A.6_M.2</v>
       </c>
-      <c r="C5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="E5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="H5" s="2" t="str">
+      <c r="C5" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D5" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E5" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F5" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G5" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H5" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="str">
-        <v/>
-      </c>
-      <c r="B6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="E6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="H6" s="2" t="str">
+      <c r="A6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="B6" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C6" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D6" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E6" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F6" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G6" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H6" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="str">
+      <c r="A7" s="4" t="str">
         <v>Controls DE</v>
       </c>
-      <c r="B7" s="2" t="str">
+      <c r="B7" s="5" t="str">
         <v>Poovarasan M</v>
       </c>
-      <c r="C7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="E7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="H7" s="2" t="str">
+      <c r="C7" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D7" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E7" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F7" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G7" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H7" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="str">
+      <c r="A8" s="4" t="str">
         <v>Phone:</v>
       </c>
-      <c r="B8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="E8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="H8" s="2" t="str">
+      <c r="B8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H8" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="str">
+      <c r="A9" s="4" t="str">
         <v>Controls ME</v>
       </c>
-      <c r="B9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="E9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="H9" s="2" t="str">
+      <c r="B9" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C9" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D9" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E9" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F9" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G9" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H9" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="str">
+      <c r="A10" s="4" t="str">
         <v>Phone:</v>
       </c>
-      <c r="B10" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C10" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D10" s="2" t="str">
-        <v/>
-      </c>
-      <c r="E10" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F10" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G10" s="2" t="str">
-        <v/>
-      </c>
-      <c r="H10" s="2" t="str">
+      <c r="B10" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C10" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D10" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E10" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F10" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G10" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H10" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="str">
-        <v/>
-      </c>
-      <c r="B11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="E11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="H11" s="2" t="str">
+      <c r="A11" s="4" t="str">
+        <v/>
+      </c>
+      <c r="B11" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C11" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D11" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E11" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F11" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G11" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H11" s="5" t="str">
         <v/>
       </c>
     </row>
@@ -846,103 +921,103 @@
       <c r="A12" s="6" t="str">
         <v>From</v>
       </c>
-      <c r="B12" s="7" t="str">
-        <v/>
-      </c>
-      <c r="C12" s="7" t="str">
-        <v/>
-      </c>
-      <c r="D12" s="7" t="str">
-        <v/>
-      </c>
-      <c r="E12" s="7" t="str">
-        <v/>
-      </c>
-      <c r="F12" s="7" t="str">
-        <v/>
-      </c>
-      <c r="G12" s="7" t="str">
+      <c r="B12" s="6" t="str">
+        <v/>
+      </c>
+      <c r="C12" s="6" t="str">
+        <v/>
+      </c>
+      <c r="D12" s="6" t="str">
+        <v/>
+      </c>
+      <c r="E12" s="6" t="str">
+        <v/>
+      </c>
+      <c r="F12" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G12" s="6" t="str">
         <v>To</v>
       </c>
-      <c r="H12" s="7" t="str">
+      <c r="H12" s="6" t="str">
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="str">
+      <c r="A13" s="7" t="str">
         <v>Device ID</v>
       </c>
-      <c r="B13" s="9" t="str">
+      <c r="B13" s="7" t="str">
         <v>Wire No.</v>
       </c>
-      <c r="C13" s="9" t="str">
+      <c r="C13" s="7" t="str">
         <v>Wire ID</v>
       </c>
-      <c r="D13" s="9" t="str">
+      <c r="D13" s="7" t="str">
         <v>Gauge/Size</v>
       </c>
-      <c r="E13" s="9" t="str">
+      <c r="E13" s="7" t="str">
         <v>Length</v>
       </c>
-      <c r="F13" s="9" t="str">
+      <c r="F13" s="7" t="str">
         <v>Device ID</v>
       </c>
-      <c r="G13" s="9" t="str">
+      <c r="G13" s="7" t="str">
         <v>To Location</v>
       </c>
-      <c r="H13" s="9" t="str">
+      <c r="H13" s="7" t="str">
         <v>Bundle Name</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="str">
+      <c r="A14" s="8" t="str">
         <v>EL</v>
       </c>
-      <c r="B14" s="11" t="str">
-        <v/>
-      </c>
-      <c r="C14" s="11" t="str">
-        <v/>
-      </c>
-      <c r="D14" s="11" t="str">
-        <v/>
-      </c>
-      <c r="E14" s="11" t="str">
-        <v/>
-      </c>
-      <c r="F14" s="11" t="str">
-        <v/>
-      </c>
-      <c r="G14" s="11" t="str">
-        <v/>
-      </c>
-      <c r="H14" s="11" t="str">
+      <c r="B14" s="8" t="str">
+        <v/>
+      </c>
+      <c r="C14" s="8" t="str">
+        <v/>
+      </c>
+      <c r="D14" s="8" t="str">
+        <v/>
+      </c>
+      <c r="E14" s="8" t="str">
+        <v/>
+      </c>
+      <c r="F14" s="8" t="str">
+        <v/>
+      </c>
+      <c r="G14" s="8" t="str">
+        <v/>
+      </c>
+      <c r="H14" s="8" t="str">
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="str">
-        <v/>
-      </c>
-      <c r="B15" s="11" t="str">
-        <v/>
-      </c>
-      <c r="C15" s="11" t="str">
-        <v/>
-      </c>
-      <c r="D15" s="11" t="str">
-        <v/>
-      </c>
-      <c r="E15" s="11" t="str">
-        <v/>
-      </c>
-      <c r="F15" s="11" t="str">
-        <v/>
-      </c>
-      <c r="G15" s="11" t="str">
-        <v/>
-      </c>
-      <c r="H15" s="11" t="str">
+      <c r="A15" s="9" t="str">
+        <v/>
+      </c>
+      <c r="B15" s="9" t="str">
+        <v/>
+      </c>
+      <c r="C15" s="9" t="str">
+        <v/>
+      </c>
+      <c r="D15" s="9" t="str">
+        <v/>
+      </c>
+      <c r="E15" s="9" t="str">
+        <v/>
+      </c>
+      <c r="F15" s="9" t="str">
+        <v/>
+      </c>
+      <c r="G15" s="9" t="str">
+        <v/>
+      </c>
+      <c r="H15" s="9" t="str">
         <v/>
       </c>
     </row>
@@ -950,129 +1025,129 @@
       <c r="A16" s="6" t="str">
         <v>EL0100:2-</v>
       </c>
-      <c r="B16" s="12" t="str">
+      <c r="B16" s="10" t="str">
         <v>-0V</v>
       </c>
-      <c r="C16" s="13" t="str">
+      <c r="C16" s="6" t="str">
         <v>WHT</v>
       </c>
-      <c r="D16" s="13" t="str">
+      <c r="D16" s="6" t="str">
         <v>16</v>
       </c>
-      <c r="E16" s="13" t="str">
+      <c r="E16" s="6" t="str">
         <v>120.0</v>
       </c>
-      <c r="F16" s="13" t="str">
+      <c r="F16" s="6" t="str">
         <v>XT0005:4</v>
       </c>
-      <c r="G16" s="13" t="str">
+      <c r="G16" s="6" t="str">
         <v>JB71 B,PNL DC PWR</v>
       </c>
-      <c r="H16" s="13" t="str">
+      <c r="H16" s="6" t="str">
         <v>EL0100</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="str">
+      <c r="A17" s="5" t="str">
         <v>EL0100:1+</v>
       </c>
-      <c r="B17" s="11" t="str">
+      <c r="B17" s="5" t="str">
         <v>FU0005</v>
       </c>
-      <c r="C17" s="11" t="str">
+      <c r="C17" s="5" t="str">
         <v>WHT</v>
       </c>
-      <c r="D17" s="11" t="str">
+      <c r="D17" s="5" t="str">
         <v>16</v>
       </c>
-      <c r="E17" s="11" t="str">
+      <c r="E17" s="5" t="str">
         <v>120.0</v>
       </c>
-      <c r="F17" s="11" t="str">
+      <c r="F17" s="5" t="str">
         <v>XT0005:2</v>
       </c>
-      <c r="G17" s="11" t="str">
+      <c r="G17" s="5" t="str">
         <v>JB71 B,PNL DC PWR</v>
       </c>
-      <c r="H17" s="11" t="str">
+      <c r="H17" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="str">
-        <v/>
-      </c>
-      <c r="B18" s="11" t="str">
-        <v/>
-      </c>
-      <c r="C18" s="11" t="str">
-        <v/>
-      </c>
-      <c r="D18" s="11" t="str">
-        <v/>
-      </c>
-      <c r="E18" s="11" t="str">
-        <v/>
-      </c>
-      <c r="F18" s="11" t="str">
-        <v/>
-      </c>
-      <c r="G18" s="11" t="str">
-        <v/>
-      </c>
-      <c r="H18" s="11" t="str">
+      <c r="A18" s="9" t="str">
+        <v/>
+      </c>
+      <c r="B18" s="9" t="str">
+        <v/>
+      </c>
+      <c r="C18" s="9" t="str">
+        <v/>
+      </c>
+      <c r="D18" s="9" t="str">
+        <v/>
+      </c>
+      <c r="E18" s="9" t="str">
+        <v/>
+      </c>
+      <c r="F18" s="9" t="str">
+        <v/>
+      </c>
+      <c r="G18" s="9" t="str">
+        <v/>
+      </c>
+      <c r="H18" s="9" t="str">
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="str">
+      <c r="A19" s="6" t="str">
         <v>EL0101:2-</v>
       </c>
-      <c r="B19" s="13" t="str">
+      <c r="B19" s="10" t="str">
         <v>-0V</v>
       </c>
-      <c r="C19" s="13" t="str">
+      <c r="C19" s="6" t="str">
         <v>WHT</v>
       </c>
-      <c r="D19" s="13" t="str">
+      <c r="D19" s="6" t="str">
         <v>16</v>
       </c>
-      <c r="E19" s="13" t="str">
+      <c r="E19" s="6" t="str">
         <v>120.0</v>
       </c>
-      <c r="F19" s="13" t="str">
+      <c r="F19" s="6" t="str">
         <v>XT0005:3</v>
       </c>
-      <c r="G19" s="13" t="str">
+      <c r="G19" s="6" t="str">
         <v>JB71 B,PNL DC PWR</v>
       </c>
-      <c r="H19" s="13" t="str">
+      <c r="H19" s="6" t="str">
         <v>EL0101</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="str">
+      <c r="A20" s="5" t="str">
         <v>EL0101:1+</v>
       </c>
-      <c r="B20" s="11" t="str">
+      <c r="B20" s="5" t="str">
         <v>FU0005</v>
       </c>
-      <c r="C20" s="11" t="str">
+      <c r="C20" s="5" t="str">
         <v>WHT</v>
       </c>
-      <c r="D20" s="11" t="str">
+      <c r="D20" s="5" t="str">
         <v>16</v>
       </c>
-      <c r="E20" s="11" t="str">
+      <c r="E20" s="5" t="str">
         <v>120.0</v>
       </c>
-      <c r="F20" s="11" t="str">
+      <c r="F20" s="5" t="str">
         <v>XT0005:1</v>
       </c>
-      <c r="G20" s="11" t="str">
+      <c r="G20" s="5" t="str">
         <v>JB71 B,PNL DC PWR</v>
       </c>
-      <c r="H20" s="11" t="str">
+      <c r="H20" s="5" t="str">
         <v/>
       </c>
     </row>

</xml_diff>